<commit_message>
Use cases 51-100: answer keys from the data, 36 new file kinds; five cards built, the rest waiting on readers and tables
</commit_message>
<xml_diff>
--- a/tests/v1/fixtures/office6m/2026-05/bank_statements/HB_B_USD_2026-04.xlsx
+++ b/tests/v1/fixtures/office6m/2026-05/bank_statements/HB_B_USD_2026-04.xlsx
@@ -649,13 +649,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
     </row>
     <row r="3">
@@ -675,13 +675,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
     </row>
     <row r="4">
@@ -701,13 +701,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
     </row>
     <row r="5">
@@ -727,13 +727,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
     </row>
     <row r="6">
@@ -753,13 +753,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
     </row>
     <row r="7">
@@ -779,13 +779,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
     </row>
     <row r="8">
@@ -805,13 +805,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
     </row>
     <row r="9">
@@ -831,13 +831,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
     </row>
     <row r="10">
@@ -857,13 +857,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
     </row>
     <row r="11">
@@ -883,13 +883,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
     </row>
     <row r="12">
@@ -909,13 +909,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
     </row>
     <row r="13">
@@ -935,13 +935,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
     </row>
     <row r="14">
@@ -961,13 +961,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
     </row>
     <row r="15">
@@ -987,13 +987,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
     </row>
     <row r="16">
@@ -1013,13 +1013,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
     </row>
     <row r="17">
@@ -1039,13 +1039,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
     </row>
     <row r="18">
@@ -1065,13 +1065,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
     </row>
     <row r="19">
@@ -1091,13 +1091,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
     </row>
     <row r="20">
@@ -1117,13 +1117,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
     </row>
     <row r="21">
@@ -1143,13 +1143,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>704314.35</v>
+        <v>706464.35</v>
       </c>
       <c r="E21" t="n">
         <v>-15272.98</v>
       </c>
       <c r="F21" t="n">
-        <v>689041.37</v>
+        <v>691191.37</v>
       </c>
     </row>
     <row r="22">
@@ -1169,13 +1169,13 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>689041.37</v>
+        <v>691191.37</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>689041.37</v>
+        <v>691191.37</v>
       </c>
     </row>
     <row r="23">
@@ -1195,13 +1195,13 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>689041.37</v>
+        <v>691191.37</v>
       </c>
       <c r="E23" t="n">
         <v>163.57</v>
       </c>
       <c r="F23" t="n">
-        <v>689204.9399999999</v>
+        <v>691354.9399999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>